<commit_message>
Fix online rows to combined form, seat VLE rows to maximise utilisation
- courses.xlsx: force split=no on online=yes rows so the VLE offering is the
  combined AB form (ES 376 / EL 162 / CV 351 / CE 451 now match every other
  course row) - no split A/B rows ship as ONLINE
- loaders: stop propagating online=yes from one row to the course's in-person
  twin rows (PROPAGATE_ONLINE_TO_DUPLICATE_ROWS = False); physical twins keep
  their classrooms
- solver: _verify/_illegal_online flag only split-form-in-ONLINE; combined dual
  rows are the intended pattern
- regen: add max_utilisation_sweep that seats combined-ONLINE rows in free
  room cells, splitting oversized rows into physical A/B halves for 80-cap
  rooms, keeping the VLE row online; report room_utilisation_pct
- sem1 settings: phase1_time_limit 1800 -> 90 (tight mode unsolvable for sem1,
  plain + postprocess path)
- regenerate both semesters: conflict-free, 0 same-day, 0 paired/mixed;
  utilisation 99.2% (sem1) and 96.8% (sem2)
</commit_message>
<xml_diff>
--- a/data/semesters/sem1/courses.xlsx
+++ b/data/semesters/sem1/courses.xlsx
@@ -1018,7 +1018,11 @@
           <t>CE100-A,CE100-B</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
@@ -1270,7 +1274,11 @@
           <t>CE100-A,CE100-B</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
@@ -1390,7 +1398,11 @@
         <v>0</v>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
@@ -1451,7 +1463,11 @@
           <t>CV200-A,CV200-B</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
@@ -1577,7 +1593,11 @@
           <t>CE200-A,CE200-B</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
@@ -1896,7 +1916,11 @@
           <t>CE200-A,CE200-B</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
@@ -2408,7 +2432,11 @@
           <t>CE300-A,CE300-B</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
@@ -2597,7 +2625,11 @@
           <t>CE300-A,CE300-B</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
@@ -2975,7 +3007,11 @@
           <t>CE400-A,CE400-B</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
@@ -3231,7 +3267,11 @@
           <t>CE400-A,CE400-B</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
@@ -3546,7 +3586,11 @@
           <t>CE400-A,CE400-B</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
@@ -4062,7 +4106,11 @@
           <t>CV100-A,CV100-B</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr"/>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="inlineStr"/>
@@ -4377,7 +4425,11 @@
           <t>CV200-A,CV200-B</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr"/>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr"/>
@@ -4503,7 +4555,11 @@
           <t>CV200-A,CV200-B</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr"/>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr"/>
@@ -4566,7 +4622,11 @@
           <t>CV200-A,CV200-B</t>
         </is>
       </c>
-      <c r="P65" t="inlineStr"/>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr"/>
@@ -5267,7 +5327,11 @@
           <t>CV300-A,CV300-B</t>
         </is>
       </c>
-      <c r="P76" t="inlineStr"/>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr"/>
@@ -5706,7 +5770,11 @@
         <v>0</v>
       </c>
       <c r="O83" t="inlineStr"/>
-      <c r="P83" t="inlineStr"/>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="inlineStr"/>
@@ -5769,7 +5837,11 @@
           <t>DS100-A</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr"/>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="inlineStr"/>
@@ -5832,7 +5904,11 @@
           <t>DS100-A</t>
         </is>
       </c>
-      <c r="P85" t="inlineStr"/>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr"/>
@@ -5895,7 +5971,11 @@
           <t>DS100-A</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr"/>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr"/>
@@ -6021,7 +6101,11 @@
           <t>DS100-A</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr"/>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q88" t="inlineStr"/>
       <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr"/>
@@ -6261,7 +6345,11 @@
           <t>DS100-A</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr"/>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q92" t="inlineStr"/>
       <c r="R92" t="inlineStr"/>
       <c r="S92" t="inlineStr"/>
@@ -6387,7 +6475,11 @@
           <t>DS200-A</t>
         </is>
       </c>
-      <c r="P94" t="inlineStr"/>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q94" t="inlineStr"/>
       <c r="R94" t="inlineStr"/>
       <c r="S94" t="inlineStr"/>
@@ -6450,7 +6542,11 @@
           <t>DS200-A</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr"/>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q95" t="inlineStr"/>
       <c r="R95" t="inlineStr"/>
       <c r="S95" t="inlineStr"/>
@@ -6828,7 +6924,11 @@
           <t>DS200-A</t>
         </is>
       </c>
-      <c r="P101" t="inlineStr"/>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q101" t="inlineStr"/>
       <c r="R101" t="inlineStr"/>
       <c r="S101" t="inlineStr"/>
@@ -7537,7 +7637,11 @@
           <t>EL200-A,EL200-B</t>
         </is>
       </c>
-      <c r="P112" t="inlineStr"/>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q112" t="inlineStr"/>
       <c r="R112" t="inlineStr"/>
       <c r="S112" t="inlineStr"/>
@@ -7600,7 +7704,11 @@
           <t>EL200-A,EL200-B</t>
         </is>
       </c>
-      <c r="P113" t="inlineStr"/>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q113" t="inlineStr"/>
       <c r="R113" t="inlineStr"/>
       <c r="S113" t="inlineStr"/>
@@ -9699,7 +9807,11 @@
           <t>ES100-A,ES100-B</t>
         </is>
       </c>
-      <c r="P146" t="inlineStr"/>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q146" t="inlineStr"/>
       <c r="R146" t="inlineStr"/>
       <c r="S146" t="inlineStr"/>
@@ -9762,7 +9874,11 @@
           <t>ES200-A,ES200-B</t>
         </is>
       </c>
-      <c r="P147" t="inlineStr"/>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q147" t="inlineStr"/>
       <c r="R147" t="inlineStr"/>
       <c r="S147" t="inlineStr"/>
@@ -9959,7 +10075,11 @@
           <t>ES200-A,ES200-B</t>
         </is>
       </c>
-      <c r="P150" t="inlineStr"/>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q150" t="inlineStr"/>
       <c r="R150" t="inlineStr"/>
       <c r="S150" t="inlineStr"/>
@@ -10022,7 +10142,11 @@
           <t>ES200-A,ES200-B</t>
         </is>
       </c>
-      <c r="P151" t="inlineStr"/>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q151" t="inlineStr"/>
       <c r="R151" t="inlineStr"/>
       <c r="S151" t="inlineStr"/>
@@ -10660,7 +10784,11 @@
           <t>ES300-A,ES300-B</t>
         </is>
       </c>
-      <c r="P161" t="inlineStr"/>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q161" t="inlineStr"/>
       <c r="R161" t="inlineStr"/>
       <c r="S161" t="inlineStr"/>
@@ -11264,7 +11392,11 @@
           <t>ES400-A,ES400-B</t>
         </is>
       </c>
-      <c r="P171" t="inlineStr"/>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q171" t="inlineStr"/>
       <c r="R171" t="inlineStr"/>
       <c r="S171" t="inlineStr"/>
@@ -11654,7 +11786,11 @@
           <t>MF100-A</t>
         </is>
       </c>
-      <c r="P177" t="inlineStr"/>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q177" t="inlineStr"/>
       <c r="R177" t="inlineStr"/>
       <c r="S177" t="inlineStr"/>
@@ -11906,7 +12042,11 @@
           <t>GL200-A,GL200-B</t>
         </is>
       </c>
-      <c r="P181" t="inlineStr"/>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q181" t="inlineStr"/>
       <c r="R181" t="inlineStr"/>
       <c r="S181" t="inlineStr"/>
@@ -12032,7 +12172,11 @@
           <t>GL200-A,GL200-B</t>
         </is>
       </c>
-      <c r="P183" t="inlineStr"/>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q183" t="inlineStr"/>
       <c r="R183" t="inlineStr"/>
       <c r="S183" t="inlineStr"/>
@@ -12095,7 +12239,11 @@
           <t>GL200-A,GL200-B</t>
         </is>
       </c>
-      <c r="P184" t="inlineStr"/>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q184" t="inlineStr"/>
       <c r="R184" t="inlineStr"/>
       <c r="S184" t="inlineStr"/>
@@ -12221,7 +12369,11 @@
           <t>GL200-A,GL200-B</t>
         </is>
       </c>
-      <c r="P186" t="inlineStr"/>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q186" t="inlineStr"/>
       <c r="R186" t="inlineStr"/>
       <c r="S186" t="inlineStr"/>
@@ -13127,7 +13279,11 @@
         <v>0</v>
       </c>
       <c r="O200" t="inlineStr"/>
-      <c r="P200" t="inlineStr"/>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q200" t="inlineStr"/>
       <c r="R200" t="inlineStr"/>
       <c r="S200" t="inlineStr"/>
@@ -13850,7 +14006,11 @@
           <t>TM100-A</t>
         </is>
       </c>
-      <c r="P211" t="inlineStr"/>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q211" t="inlineStr"/>
       <c r="R211" t="inlineStr"/>
       <c r="S211" t="inlineStr"/>
@@ -15436,7 +15596,11 @@
         <v>0</v>
       </c>
       <c r="O235" t="inlineStr"/>
-      <c r="P235" t="inlineStr"/>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q235" t="inlineStr"/>
       <c r="R235" t="inlineStr"/>
       <c r="S235" t="inlineStr"/>
@@ -15493,7 +15657,11 @@
         <v>0</v>
       </c>
       <c r="O236" t="inlineStr"/>
-      <c r="P236" t="inlineStr"/>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q236" t="inlineStr"/>
       <c r="R236" t="inlineStr"/>
       <c r="S236" t="inlineStr"/>
@@ -18940,7 +19108,11 @@
           <t>MF100-A</t>
         </is>
       </c>
-      <c r="P289" t="inlineStr"/>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q289" t="inlineStr"/>
       <c r="R289" t="inlineStr"/>
       <c r="S289" t="inlineStr"/>
@@ -19192,7 +19364,11 @@
           <t>MF100-A</t>
         </is>
       </c>
-      <c r="P293" t="inlineStr"/>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q293" t="inlineStr"/>
       <c r="R293" t="inlineStr"/>
       <c r="S293" t="inlineStr"/>
@@ -19255,7 +19431,11 @@
           <t>MF100-A</t>
         </is>
       </c>
-      <c r="P294" t="inlineStr"/>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q294" t="inlineStr"/>
       <c r="R294" t="inlineStr"/>
       <c r="S294" t="inlineStr"/>
@@ -19444,7 +19624,11 @@
           <t>TM100-A</t>
         </is>
       </c>
-      <c r="P297" t="inlineStr"/>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q297" t="inlineStr"/>
       <c r="R297" t="inlineStr"/>
       <c r="S297" t="inlineStr"/>
@@ -19507,7 +19691,11 @@
           <t>TM100-A</t>
         </is>
       </c>
-      <c r="P298" t="inlineStr"/>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q298" t="inlineStr"/>
       <c r="R298" t="inlineStr"/>
       <c r="S298" t="inlineStr"/>
@@ -19570,7 +19758,11 @@
           <t>TM100-A</t>
         </is>
       </c>
-      <c r="P299" t="inlineStr"/>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="Q299" t="inlineStr"/>
       <c r="R299" t="inlineStr"/>
       <c r="S299" t="inlineStr"/>

</xml_diff>